<commit_message>
adding IPC netlist and fixed stackup file due to another typo
</commit_message>
<xml_diff>
--- a/stackup-K2-6lyr-FR408HR-10_MAR_2026.xlsx
+++ b/stackup-K2-6lyr-FR408HR-10_MAR_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\tmp\hw-k2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1D3DF6A-82DE-4AAA-AD09-519CE10D1299}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E823E90C-E1B7-4432-80EC-D95FF4293D7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="31920" xr2:uid="{80DBAC24-F6F6-4201-9AF3-F62C14734A8F}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="29010" windowHeight="31785" xr2:uid="{80DBAC24-F6F6-4201-9AF3-F62C14734A8F}"/>
   </bookViews>
   <sheets>
     <sheet name="Stackup" sheetId="23" r:id="rId1"/>
@@ -736,80 +736,80 @@
     <xf numFmtId="164" fontId="20" fillId="6" borderId="7" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="167" fontId="19" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="20" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="20" fillId="5" borderId="7" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="20" fillId="6" borderId="7" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="19" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="20" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="14" fontId="14" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="14" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="167" fontId="19" fillId="4" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="20" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="20" fillId="5" borderId="7" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="20" fillId="6" borderId="7" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="19" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="20" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1164,13 +1164,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:12" ht="28.5" customHeight="1">
-      <c r="B2" s="50" t="s">
+      <c r="B2" s="72" t="s">
         <v>30</v>
       </c>
-      <c r="C2" s="50"/>
-      <c r="D2" s="50"/>
-      <c r="E2" s="50"/>
-      <c r="F2" s="50"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
+      <c r="F2" s="72"/>
       <c r="G2" s="10"/>
       <c r="H2" s="10"/>
       <c r="I2" s="10"/>
@@ -1192,145 +1192,145 @@
       <c r="L3" s="12"/>
     </row>
     <row r="4" spans="2:12">
-      <c r="B4" s="48" t="s">
+      <c r="B4" s="68" t="s">
         <v>25</v>
       </c>
-      <c r="C4" s="48"/>
-      <c r="D4" s="49" t="s">
+      <c r="C4" s="68"/>
+      <c r="D4" s="70" t="s">
         <v>58</v>
       </c>
-      <c r="E4" s="49"/>
-      <c r="F4" s="49"/>
+      <c r="E4" s="70"/>
+      <c r="F4" s="70"/>
       <c r="J4" s="12"/>
       <c r="K4" s="12"/>
     </row>
     <row r="5" spans="2:12">
-      <c r="B5" s="48" t="s">
+      <c r="B5" s="68" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="48"/>
-      <c r="D5" s="49" t="s">
+      <c r="C5" s="68"/>
+      <c r="D5" s="70" t="s">
         <v>42</v>
       </c>
-      <c r="E5" s="49"/>
-      <c r="F5" s="49"/>
+      <c r="E5" s="70"/>
+      <c r="F5" s="70"/>
       <c r="J5" s="12"/>
       <c r="K5" s="12"/>
     </row>
     <row r="6" spans="2:12">
-      <c r="B6" s="48" t="s">
+      <c r="B6" s="68" t="s">
         <v>59</v>
       </c>
-      <c r="C6" s="48"/>
-      <c r="D6" s="49" t="s">
+      <c r="C6" s="68"/>
+      <c r="D6" s="70" t="s">
         <v>60</v>
       </c>
-      <c r="E6" s="49"/>
-      <c r="F6" s="49"/>
+      <c r="E6" s="70"/>
+      <c r="F6" s="70"/>
       <c r="J6" s="12"/>
       <c r="K6" s="12"/>
     </row>
     <row r="7" spans="2:12">
-      <c r="B7" s="48" t="s">
+      <c r="B7" s="68" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="48"/>
-      <c r="D7" s="49" t="s">
+      <c r="C7" s="68"/>
+      <c r="D7" s="70" t="s">
         <v>43</v>
       </c>
-      <c r="E7" s="49"/>
-      <c r="F7" s="49"/>
+      <c r="E7" s="70"/>
+      <c r="F7" s="70"/>
       <c r="J7" s="12"/>
       <c r="K7" s="12"/>
     </row>
     <row r="8" spans="2:12">
-      <c r="B8" s="48" t="s">
+      <c r="B8" s="68" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="48"/>
-      <c r="D8" s="49" t="s">
+      <c r="C8" s="68"/>
+      <c r="D8" s="70" t="s">
         <v>44</v>
       </c>
-      <c r="E8" s="49"/>
-      <c r="F8" s="49"/>
+      <c r="E8" s="70"/>
+      <c r="F8" s="70"/>
       <c r="J8" s="12"/>
       <c r="K8" s="12"/>
     </row>
     <row r="9" spans="2:12">
-      <c r="B9" s="48" t="s">
+      <c r="B9" s="68" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="48"/>
-      <c r="D9" s="49" t="s">
+      <c r="C9" s="68"/>
+      <c r="D9" s="70" t="s">
         <v>45</v>
       </c>
-      <c r="E9" s="49"/>
-      <c r="F9" s="49"/>
+      <c r="E9" s="70"/>
+      <c r="F9" s="70"/>
       <c r="J9" s="12"/>
       <c r="K9" s="12"/>
     </row>
     <row r="10" spans="2:12">
-      <c r="B10" s="48" t="s">
+      <c r="B10" s="68" t="s">
         <v>18</v>
       </c>
-      <c r="C10" s="48"/>
-      <c r="D10" s="49" t="s">
+      <c r="C10" s="68"/>
+      <c r="D10" s="70" t="s">
         <v>47</v>
       </c>
-      <c r="E10" s="49"/>
-      <c r="F10" s="49"/>
+      <c r="E10" s="70"/>
+      <c r="F10" s="70"/>
       <c r="J10" s="12"/>
       <c r="K10" s="12"/>
     </row>
     <row r="11" spans="2:12">
-      <c r="B11" s="48" t="s">
+      <c r="B11" s="68" t="s">
         <v>56</v>
       </c>
-      <c r="C11" s="48"/>
-      <c r="D11" s="49" t="s">
+      <c r="C11" s="68"/>
+      <c r="D11" s="70" t="s">
         <v>57</v>
       </c>
-      <c r="E11" s="49"/>
-      <c r="F11" s="49"/>
+      <c r="E11" s="70"/>
+      <c r="F11" s="70"/>
       <c r="J11" s="12"/>
       <c r="K11" s="12"/>
     </row>
     <row r="12" spans="2:12" ht="26.25" customHeight="1">
-      <c r="B12" s="48" t="s">
+      <c r="B12" s="68" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="48"/>
-      <c r="D12" s="51" t="s">
+      <c r="C12" s="68"/>
+      <c r="D12" s="71" t="s">
         <v>46</v>
       </c>
-      <c r="E12" s="49"/>
-      <c r="F12" s="49"/>
+      <c r="E12" s="70"/>
+      <c r="F12" s="70"/>
       <c r="J12" s="12"/>
       <c r="K12" s="12"/>
     </row>
     <row r="13" spans="2:12">
-      <c r="B13" s="48" t="s">
+      <c r="B13" s="68" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="48"/>
-      <c r="D13" s="52">
+      <c r="C13" s="68"/>
+      <c r="D13" s="69">
         <v>46091</v>
       </c>
-      <c r="E13" s="49"/>
-      <c r="F13" s="49"/>
+      <c r="E13" s="70"/>
+      <c r="F13" s="70"/>
       <c r="J13" s="12"/>
       <c r="K13" s="12"/>
     </row>
     <row r="14" spans="2:12">
-      <c r="B14" s="48" t="s">
+      <c r="B14" s="68" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="48"/>
-      <c r="D14" s="49" t="s">
+      <c r="C14" s="68"/>
+      <c r="D14" s="70" t="s">
         <v>48</v>
       </c>
-      <c r="E14" s="49"/>
-      <c r="F14" s="49"/>
+      <c r="E14" s="70"/>
+      <c r="F14" s="70"/>
       <c r="J14" s="12"/>
       <c r="K14" s="12"/>
     </row>
@@ -1343,69 +1343,69 @@
     </row>
     <row r="16" spans="2:12" ht="14.45" customHeight="1"/>
     <row r="17" spans="2:14">
-      <c r="B17" s="53" t="s">
+      <c r="B17" s="63" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="53" t="s">
+      <c r="C17" s="63" t="s">
         <v>10</v>
       </c>
-      <c r="D17" s="53" t="s">
+      <c r="D17" s="63" t="s">
         <v>17</v>
       </c>
-      <c r="E17" s="53" t="s">
+      <c r="E17" s="63" t="s">
         <v>20</v>
       </c>
-      <c r="F17" s="53" t="s">
+      <c r="F17" s="63" t="s">
         <v>22</v>
       </c>
-      <c r="G17" s="53"/>
-      <c r="H17" s="58" t="s">
+      <c r="G17" s="63"/>
+      <c r="H17" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="I17" s="59"/>
-      <c r="J17" s="53" t="s">
+      <c r="I17" s="58"/>
+      <c r="J17" s="63" t="s">
         <v>27</v>
       </c>
-      <c r="K17" s="53" t="s">
+      <c r="K17" s="63" t="s">
         <v>29</v>
       </c>
       <c r="L17" s="64" t="s">
         <v>28</v>
       </c>
-      <c r="M17" s="54" t="s">
+      <c r="M17" s="55" t="s">
         <v>40</v>
       </c>
-      <c r="N17" s="55"/>
+      <c r="N17" s="56"/>
     </row>
     <row r="18" spans="2:14">
-      <c r="B18" s="53"/>
-      <c r="C18" s="53"/>
-      <c r="D18" s="53"/>
-      <c r="E18" s="53"/>
-      <c r="F18" s="53"/>
-      <c r="G18" s="53"/>
-      <c r="H18" s="60"/>
-      <c r="I18" s="61"/>
-      <c r="J18" s="53"/>
-      <c r="K18" s="53"/>
-      <c r="L18" s="53"/>
-      <c r="M18" s="56" t="s">
+      <c r="B18" s="63"/>
+      <c r="C18" s="63"/>
+      <c r="D18" s="63"/>
+      <c r="E18" s="63"/>
+      <c r="F18" s="63"/>
+      <c r="G18" s="63"/>
+      <c r="H18" s="59"/>
+      <c r="I18" s="60"/>
+      <c r="J18" s="63"/>
+      <c r="K18" s="63"/>
+      <c r="L18" s="63"/>
+      <c r="M18" s="67" t="s">
         <v>13</v>
       </c>
-      <c r="N18" s="56"/>
+      <c r="N18" s="67"/>
     </row>
     <row r="19" spans="2:14">
-      <c r="B19" s="53"/>
-      <c r="C19" s="53"/>
-      <c r="D19" s="53"/>
-      <c r="E19" s="53"/>
-      <c r="F19" s="53"/>
-      <c r="G19" s="53"/>
-      <c r="H19" s="62"/>
-      <c r="I19" s="63"/>
-      <c r="J19" s="53"/>
-      <c r="K19" s="53"/>
-      <c r="L19" s="53"/>
+      <c r="B19" s="63"/>
+      <c r="C19" s="63"/>
+      <c r="D19" s="63"/>
+      <c r="E19" s="63"/>
+      <c r="F19" s="63"/>
+      <c r="G19" s="63"/>
+      <c r="H19" s="61"/>
+      <c r="I19" s="62"/>
+      <c r="J19" s="63"/>
+      <c r="K19" s="63"/>
+      <c r="L19" s="63"/>
       <c r="M19" s="6" t="s">
         <v>39</v>
       </c>
@@ -1414,10 +1414,10 @@
       </c>
     </row>
     <row r="20" spans="2:14">
-      <c r="B20" s="53"/>
-      <c r="C20" s="53"/>
-      <c r="D20" s="53"/>
-      <c r="E20" s="53"/>
+      <c r="B20" s="63"/>
+      <c r="C20" s="63"/>
+      <c r="D20" s="63"/>
+      <c r="E20" s="63"/>
       <c r="F20" s="6" t="s">
         <v>21</v>
       </c>
@@ -1430,9 +1430,9 @@
       <c r="I20" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="J20" s="53"/>
-      <c r="K20" s="53"/>
-      <c r="L20" s="53"/>
+      <c r="J20" s="63"/>
+      <c r="K20" s="63"/>
+      <c r="L20" s="63"/>
       <c r="M20" s="6" t="s">
         <v>31</v>
       </c>
@@ -1453,7 +1453,7 @@
       <c r="E21" s="30"/>
       <c r="F21" s="30"/>
       <c r="G21" s="30"/>
-      <c r="H21" s="67">
+      <c r="H21" s="48">
         <v>0.5</v>
       </c>
       <c r="I21" s="30"/>
@@ -1480,7 +1480,7 @@
         <v>51</v>
       </c>
       <c r="G22" s="23"/>
-      <c r="H22" s="68">
+      <c r="H22" s="49">
         <v>1.45</v>
       </c>
       <c r="I22" s="23"/>
@@ -1509,7 +1509,7 @@
       </c>
       <c r="F23" s="33"/>
       <c r="G23" s="33"/>
-      <c r="H23" s="69">
+      <c r="H23" s="50">
         <v>2.996</v>
       </c>
       <c r="I23" s="33"/>
@@ -1536,7 +1536,7 @@
         <v>3</v>
       </c>
       <c r="G24" s="23"/>
-      <c r="H24" s="68">
+      <c r="H24" s="49">
         <v>1.4</v>
       </c>
       <c r="I24" s="23"/>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="F25" s="38"/>
       <c r="G25" s="38"/>
-      <c r="H25" s="70">
+      <c r="H25" s="51">
         <v>5</v>
       </c>
       <c r="I25" s="38"/>
@@ -1588,7 +1588,7 @@
         <v>3</v>
       </c>
       <c r="G26" s="23"/>
-      <c r="H26" s="68">
+      <c r="H26" s="49">
         <v>1.4</v>
       </c>
       <c r="I26" s="23"/>
@@ -1612,12 +1612,12 @@
       <c r="D27" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="E27" s="72" t="s">
+      <c r="E27" s="53" t="s">
         <v>52</v>
       </c>
       <c r="F27" s="35"/>
       <c r="G27" s="35"/>
-      <c r="H27" s="69">
+      <c r="H27" s="50">
         <f>(36.072-H28)/2</f>
         <v>7.5360000000000014</v>
       </c>
@@ -1643,7 +1643,7 @@
       </c>
       <c r="F28" s="38"/>
       <c r="G28" s="38"/>
-      <c r="H28" s="70">
+      <c r="H28" s="51">
         <v>21</v>
       </c>
       <c r="I28" s="38"/>
@@ -1667,12 +1667,12 @@
       <c r="D29" s="35" t="s">
         <v>45</v>
       </c>
-      <c r="E29" s="72" t="s">
+      <c r="E29" s="53" t="s">
         <v>52</v>
       </c>
       <c r="F29" s="35"/>
       <c r="G29" s="35"/>
-      <c r="H29" s="69">
+      <c r="H29" s="50">
         <f>H27</f>
         <v>7.5360000000000014</v>
       </c>
@@ -1696,7 +1696,7 @@
         <v>3</v>
       </c>
       <c r="G30" s="23"/>
-      <c r="H30" s="68">
+      <c r="H30" s="49">
         <v>1.4</v>
       </c>
       <c r="I30" s="23"/>
@@ -1721,7 +1721,7 @@
       </c>
       <c r="F31" s="42"/>
       <c r="G31" s="42"/>
-      <c r="H31" s="70">
+      <c r="H31" s="51">
         <v>5</v>
       </c>
       <c r="I31" s="42"/>
@@ -1748,7 +1748,7 @@
         <v>3</v>
       </c>
       <c r="G32" s="23"/>
-      <c r="H32" s="68">
+      <c r="H32" s="49">
         <v>1.4</v>
       </c>
       <c r="I32" s="23"/>
@@ -1773,7 +1773,7 @@
       </c>
       <c r="F33" s="33"/>
       <c r="G33" s="33"/>
-      <c r="H33" s="69">
+      <c r="H33" s="50">
         <v>2.996</v>
       </c>
       <c r="I33" s="33"/>
@@ -1800,7 +1800,7 @@
         <v>51</v>
       </c>
       <c r="G34" s="23"/>
-      <c r="H34" s="68">
+      <c r="H34" s="49">
         <f>H22</f>
         <v>1.45</v>
       </c>
@@ -1829,7 +1829,7 @@
       <c r="E35" s="32"/>
       <c r="F35" s="32"/>
       <c r="G35" s="32"/>
-      <c r="H35" s="71">
+      <c r="H35" s="52">
         <f>H21</f>
         <v>0.5</v>
       </c>
@@ -1898,42 +1898,42 @@
     </row>
     <row r="40" spans="2:14">
       <c r="B40" s="15"/>
-      <c r="C40" s="57"/>
-      <c r="D40" s="57"/>
-      <c r="E40" s="57"/>
-      <c r="F40" s="57"/>
-      <c r="G40" s="57"/>
-      <c r="H40" s="57"/>
-      <c r="I40" s="57"/>
-      <c r="J40" s="57"/>
-      <c r="K40" s="57"/>
-      <c r="L40" s="57"/>
+      <c r="C40" s="54"/>
+      <c r="D40" s="54"/>
+      <c r="E40" s="54"/>
+      <c r="F40" s="54"/>
+      <c r="G40" s="54"/>
+      <c r="H40" s="54"/>
+      <c r="I40" s="54"/>
+      <c r="J40" s="54"/>
+      <c r="K40" s="54"/>
+      <c r="L40" s="54"/>
     </row>
     <row r="41" spans="2:14">
       <c r="B41" s="15"/>
-      <c r="C41" s="57"/>
-      <c r="D41" s="57"/>
-      <c r="E41" s="57"/>
-      <c r="F41" s="57"/>
-      <c r="G41" s="57"/>
-      <c r="H41" s="57"/>
-      <c r="I41" s="57"/>
-      <c r="J41" s="57"/>
-      <c r="K41" s="57"/>
-      <c r="L41" s="57"/>
+      <c r="C41" s="54"/>
+      <c r="D41" s="54"/>
+      <c r="E41" s="54"/>
+      <c r="F41" s="54"/>
+      <c r="G41" s="54"/>
+      <c r="H41" s="54"/>
+      <c r="I41" s="54"/>
+      <c r="J41" s="54"/>
+      <c r="K41" s="54"/>
+      <c r="L41" s="54"/>
     </row>
     <row r="42" spans="2:14">
       <c r="B42" s="15"/>
-      <c r="C42" s="57"/>
-      <c r="D42" s="57"/>
-      <c r="E42" s="57"/>
-      <c r="F42" s="57"/>
-      <c r="G42" s="57"/>
-      <c r="H42" s="57"/>
-      <c r="I42" s="57"/>
-      <c r="J42" s="57"/>
-      <c r="K42" s="57"/>
-      <c r="L42" s="57"/>
+      <c r="C42" s="54"/>
+      <c r="D42" s="54"/>
+      <c r="E42" s="54"/>
+      <c r="F42" s="54"/>
+      <c r="G42" s="54"/>
+      <c r="H42" s="54"/>
+      <c r="I42" s="54"/>
+      <c r="J42" s="54"/>
+      <c r="K42" s="54"/>
+      <c r="L42" s="54"/>
     </row>
     <row r="43" spans="2:14">
       <c r="B43" s="15"/>
@@ -1945,6 +1945,34 @@
     </row>
   </sheetData>
   <mergeCells count="39">
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="D6:F6"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D4:F4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="D5:F5"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="D7:F7"/>
+    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="D8:F8"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="D11:F11"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="D12:F12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D13:F13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="D14:F14"/>
+    <mergeCell ref="B17:B20"/>
+    <mergeCell ref="C17:C20"/>
+    <mergeCell ref="D17:D20"/>
+    <mergeCell ref="E17:E20"/>
+    <mergeCell ref="F17:G19"/>
     <mergeCell ref="C41:L41"/>
     <mergeCell ref="C42:L42"/>
     <mergeCell ref="M17:N17"/>
@@ -1956,34 +1984,6 @@
     <mergeCell ref="B37:G37"/>
     <mergeCell ref="C40:L40"/>
     <mergeCell ref="M18:N18"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="D13:F13"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="D14:F14"/>
-    <mergeCell ref="B17:B20"/>
-    <mergeCell ref="C17:C20"/>
-    <mergeCell ref="D17:D20"/>
-    <mergeCell ref="E17:E20"/>
-    <mergeCell ref="F17:G19"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="B11:C11"/>
-    <mergeCell ref="D11:F11"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="D12:F12"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="D7:F7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="D8:F8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="D6:F6"/>
-    <mergeCell ref="B2:F2"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="D4:F4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="D5:F5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>